<commit_message>
Changes in de-bugging drill and exercise question tab.
</commit_message>
<xml_diff>
--- a/frontend/src/app/candidate-dashboard/round-2-learning/exercise-question/questions/exercise-questions.xlsx
+++ b/frontend/src/app/candidate-dashboard/round-2-learning/exercise-question/questions/exercise-questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Karat\karat-prep-assistant\frontend\src\app\candidate-dashboard\round-2-learning\exercise-question\questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D769DF-0E5A-49A7-825E-178E7FA4DDA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22493FD2-F88A-44F8-9A76-8C260D277A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>QuestionNo</t>
   </si>
@@ -32,12 +32,6 @@
   </si>
   <si>
     <t>First Non Repeating Element</t>
-  </si>
-  <si>
-    <t>Two Sum</t>
-  </si>
-  <si>
-    <t>Find Duplicate</t>
   </si>
   <si>
     <t>import java.util.*;
@@ -61,43 +55,412 @@
 }</t>
   </si>
   <si>
-    <t>import java.util.*;
-public class Main {
-    public static int[] twoSum(int[] arr, int target) {
-        Map&lt;Integer, Integer&gt; seen = new HashMap&lt;&gt;();
-        for (int i = 0; i &lt; arr.length; i++) {
-            int needed = target - arr[i];
-            if (seen.containsKey(needed)) {
-                return new int[]{seen.get(needed), i};
-            }
-            seen.put(arr[i], i);
-        }
-        return new int[]{-1, -1};
-    }
-    public static void main(String[] args) {
-        int[] arr = {2, 7, 11, 15};
-        int target = 9;
-        System.out.println(
-            Arrays.toString(twoSum(arr, target))
-        );
-    }
-}</t>
-  </si>
-  <si>
-    <t>import java.util.*;
-public class Main {
-    public static int findDuplicate(int[] arr) {
-        Set&lt;Integer&gt; seen = new HashSet&lt;&gt;();
-        for (int num : arr) {
-            if (!seen.add(num)) {
-                return num;
+    <t>Payment Transaction Monitoring</t>
+  </si>
+  <si>
+    <t>/*
+ This code implements a payment transaction monitoring system.
+ It tracks accounts and their transactions, computes current balances,
+ and provides analytics such as average transaction amount per account.
+ Definitions:
+ - An account has a unique accountid and an owner name.
+ - A transaction represents money moving in or out of an account.
+ - CREDIT increases account balance.
+ - DEBIT decreases account balance.
+ AccountManager manages accounts and transactions.
+ getBalance should add CREDIT amounts and subtract DEBIT amounts.
+ getAverageTransactionAmountByAccount should return the average absolute
+ transaction amount per account, excluding accounts with no transactions.
+*/
+import java.util.*;
+import org.junit.Assert;
+import org.junit.Test;
+enum TransactionType {
+    CREDIT,
+    DEBIT
+}
+class Account {
+    int accountid;
+    String ownerName;
+    Account(int accountid, String ownerName) {
+        this.accountid = accountid;
+        this.ownerName = ownerName;
+    }
+}
+class Transaction {
+    int transactionid;
+    int accountid;
+    TransactionType type;
+    double amount; // Always positive in inputs
+    long timestampSec; // Unix-style seconds (monotonic for tests)
+    Transaction(int transactionid, int accountid, TransactionType type, double amount, long timestampSec) {
+        this.transactionid = transactionid;
+        this.accountid = accountid;
+        this.type = type;
+        this.amount = amount;
+        this.timestampSec = timestampSec;
+    }
+}
+class AccountManager {
+    Map&lt;Integer, Account&gt; accounts = new HashMap&lt;&gt;();
+    List&lt;Transaction&gt; transactions = new ArrayList&lt;&gt;();
+    void addAccount(Account account) {
+        accounts.put(account.accountid, account);
+    }
+    // Returns the current balance for the given accountid.
+    double getBalance(int accountid) {
+        double balance = 0.0;
+        for (Transaction tx : transactions) {
+            if (tx.accountid == accountid) {
+                if (tx.type == TransactionType.CREDIT) {
+                    balance += tx.amount;
+                }
             }
         }
-        return -1;
-    }
-    public static void main(String[] args) {
-        int[] arr = {1, 3, 4, 2, 2};
-        System.out.println(findDuplicate(arr));
+        return balance;
+    }
+}
+class Solution {
+    public static void callMethod() {
+        System.out.println("Inside call Test Method.");
+        testGetBalance_basic();
+        testGetBalance_multipleAccounts();
+        testGetAverageTransactionAmountByAccount();
+        System.out.println("All tests passed.");
+    }
+    private static void assertAlmost(double expected, double actual, double eps) {
+        Assert.assertTrue("Expected " + expected + " but got " + actual,
+                Math.abs(expected - actual) &lt;= eps);
+    }
+    public static void testGetBalance_basic() {
+        System.out.println("Running testGetBalance basic");
+        AccountManager mgr = new AccountManager();
+        mgr.addAccount(new Account(1, "Alice"));
+        mgr.addTransaction(new Transaction(101, 1, TransactionType.CREDIT, 100.0, 1000));
+        mgr.addTransaction(new Transaction(102, 1, TransactionType.DEBIT, 30.0, 1010));
+        mgr.addTransaction(new Transaction(103, 1, TransactionType.DEBIT, 20.0, 1020));
+        mgr.addTransaction(new Transaction(104, 1, TransactionType.CREDIT, 10.0, 1030));
+        assertAlmost(60.0, mgr.getBalance(1), 0.0001);
+    }
+    public static void testGetBalance_multipleAccounts() {
+        System.out.println("Running testGetBalance multipleAccounts");
+        AccountManager mgr = new AccountManager();
+        mgr.addAccount(new Account(1, "Alice"));
+        mgr.addAccount(new Account(2, "Bob"));
+        mgr.addTransaction(new Transaction(201, 1, TransactionType.CREDIT, 50.0, 2000));
+        mgr.addTransaction(new Transaction(202, 2, TransactionType.CREDIT, 80.0, 2005));
+        mgr.addTransaction(new Transaction(203, 1, TransactionType.DEBIT, 10.0, 2010));
+        mgr.addTransaction(new Transaction(204, 2, TransactionType.DEBIT, 5.5, 2015));
+        mgr.addTransaction(new Transaction(205, 2, TransactionType.DEBIT, 14.5, 2020));
+        assertAlmost(40.0, mgr.getBalance(1), 0.0001);
+        assertAlmost(60.0, mgr.getBalance(2), 0.0001);
+    }
+    public static void testGetAverageTransactionAmountByAccount() {
+        System.out.println("Running testGetAverage Transaction Amount ByAccount");
+        AccountManager mgr = new AccountManager();
+        mgr.addAccount(new Account(1, "Alice"));
+        mgr.addAccount(new Account(2, "Bob"));
+        mgr.addAccount(new Account(3, "Charlie")); // no transactions
+        mgr.addTransaction(new Transaction(101, 1, TransactionType.CREDIT, 100.0, 1000));
+        mgr.addTransaction(new Transaction(102, 1, TransactionType.DEBIT, 30.0, 1010));
+        mgr.addTransaction(new Transaction(103, 1, TransactionType.DEBIT, 20.0, 1020));
+        mgr.addTransaction(new Transaction(104, 1, TransactionType.CREDIT, 10.0, 1030));
+        mgr.addTransaction(new Transaction(201, 2, TransactionType.CREDIT, 80.0, 2005));
+        mgr.addTransaction(new Transaction(202, 2, TransactionType.DEBIT, 5.5, 2015));
+        mgr.addTransaction(new Transaction(203, 2, TransactionType.DEBIT, 14.5, 2020));
+        Map&lt;Integer, Double&gt; avg = mgr.getAverageTransactionAmountByAccount();
+        assertAlmost(40.0, avg.get(1), 0.0001);
+        assertAlmost(33.3333, avg.get(2), 0.0001);
+        Assert.assertFalse(avg.containsKey(3));
+    }
+}
+public class MainTest{
+    @Test
+    public void testMethod(){
+        Solution.callMethod();
+    }
+}</t>
+  </si>
+  <si>
+    <t>E-Commerce Order Management</t>
+  </si>
+  <si>
+    <t>/*
+ *
+ * E-Commerce Order Management System
+ *
+ * The system tracks customers and their orders.
+ *
+ * Definitions:
+ * - A customer has a unique customerId and name.
+ * - An order belongs to a customer and contains an amount.
+ * - COMPLETED orders contribute to revenue.
+ * - CANCELLED orders should not contribute to revenue.
+ * - getTotalRevenueByCustomer should return the total completed
+ *   order amount for each customer.
+ * - getOrderCount should return the number of completed orders
+ *   for the given customer.
+ *
+ */
+import java.util.*;
+import org.junit.Assert;
+import org.junit.Test;
+enum OrderStatus {
+    COMPLETED,
+    CANCELLED
+}
+class Customer {
+    int customerId;
+    String name;
+    Customer(int customerId, String name) {
+        this.customerId = customerId;
+        this.name = name;
+    }
+}
+class Order {
+    int orderId;
+    int customerId;
+    double amount;
+    OrderStatus status;
+    Order(int orderId, int customerId, double amount, OrderStatus status) {
+        this.orderId = orderId;
+        this.customerId = customerId;
+        this.amount = amount;
+        this.status = status;
+    }
+}
+class OrderManager {
+    Map&lt;Integer, Customer&gt; customers = new HashMap&lt;&gt;();
+    List&lt;Order&gt; orders = new ArrayList&lt;&gt;();
+    void addCustomer(Customer customer) {
+        customers.put(customer.customerId, customer);
+    }
+    // Returns the number of completed orders for a customer.
+    int getOrderCount(int customerId) {
+        int count = 0;
+        for (Order order : orders) {
+            if (order.customerId == customerId) {
+                count++;
+            }
+        }
+        return count;
+    }
+    // Returns total completed revenue grouped by customer.
+    Map&lt;Integer, Double&gt; getTotalRevenueByCustomer() {
+        Map&lt;Integer, Double&gt; revenue = new HashMap&lt;&gt;();
+        for (Order order : orders) {
+            if (order.status == OrderStatus.COMPLETED) {
+                revenue.put(order.customerId, order.amount);
+            }
+        }
+        return revenue;
+    }
+}
+class Solution {
+    public static void callMethod() {
+        testOrderCount();
+        testRevenueByCustomer();
+        System.out.println("All tests passed.");
+    }
+    public static void testOrderCount() {
+        OrderManager manager = new OrderManager();
+        manager.addCustomer(new Customer(1, "Alice"));
+        manager.addCustomer(new Customer(2, "Bob"));
+        manager.addOrder(
+                new Order(101, 1, 100.0, OrderStatus.COMPLETED)
+        );
+        manager.addOrder(
+                new Order(102, 1, 50.0, OrderStatus.CANCELLED)
+        );
+        manager.addOrder(
+                new Order(103, 1, 75.0, OrderStatus.COMPLETED)
+        );
+        manager.addOrder(
+                new Order(104, 2, 200.0, OrderStatus.COMPLETED)
+        );
+        Assert.assertEquals(2, manager.getOrderCount(1));
+        Assert.assertEquals(1, manager.getOrderCount(2));
+    }
+    public static void testRevenueByCustomer() {
+        OrderManager manager = new OrderManager();
+        manager.addCustomer(new Customer(1, "Alice"));
+        manager.addCustomer(new Customer(2, "Bob"));
+        manager.addOrder(
+                new Order(101, 1, 100.0, OrderStatus.COMPLETED)
+        );
+        manager.addOrder(
+                new Order(102, 1, 50.0, OrderStatus.COMPLETED)
+        );
+        manager.addOrder(
+                new Order(103, 1, 25.0, OrderStatus.CANCELLED)
+        );
+        manager.addOrder(
+                new Order(104, 2, 200.0, OrderStatus.COMPLETED)
+        );
+        Map&lt;Integer, Double&gt; revenue =
+                manager.getTotalRevenueByCustomer();
+        Assert.assertEquals(150.0, revenue.get(1), 0.0001);
+        Assert.assertEquals(200.0, revenue.get(2), 0.0001);
+    }
+}
+public class MainTest {
+    @Test
+    public void testMethod() {
+        Solution.callMethod();
+    }
+}</t>
+  </si>
+  <si>
+    <t>Product Inventory and Stock Management</t>
+  </si>
+  <si>
+    <t>/*
+ *
+ * Product Inventory Management System
+ *
+ * The system tracks products and inventory movements.
+ *
+ * Definitions:
+ * - A product has a unique productId, name and price.
+ * - RESTOCK increases the available quantity.
+ * - SALE decreases the available quantity.
+ * - getCurrentStock should return the current quantity of a product.
+ * - getInventoryValue should return the total value of all
+ *   currently available products.
+ * - Inventory value = current stock * product price.
+ *
+ */
+import java.util.*;
+import org.junit.Assert;
+import org.junit.Test;
+enum MovementType {
+    RESTOCK,
+    SALE
+}
+class Product {
+    int productId;
+    String name;
+    double price;
+    Product(int productId, String name, double price) {
+        this.productId = productId;
+        this.name = name;
+        this.price = price;
+    }
+}
+class InventoryMovement {
+    int productId;
+    MovementType type;
+    int quantity;
+    InventoryMovement(int productId, MovementType type, int quantity) {
+        this.productId = productId;
+        this.type = type;
+        this.quantity = quantity;
+    }
+}
+class InventoryManager {
+    Map&lt;Integer, Product&gt; products = new HashMap&lt;&gt;();
+    List&lt;InventoryMovement&gt; movements = new ArrayList&lt;&gt;();
+    void addProduct(Product product) {
+        products.put(product.productId, product);
+    }
+    // Returns the current stock for the given product.
+    int getCurrentStock(int productId) {
+        int stock = 0;
+        for (InventoryMovement movement : movements) {
+            if (movement.productId == productId) {
+                if (movement.type == MovementType.RESTOCK) {
+                    stock += movement.quantity;
+                }
+            }
+        }
+        return stock;
+    }
+    // Returns the total value of all available inventory.
+    double getInventoryValue() {
+        double value = 0.0;
+        for (Product product : products.values()) {
+            value += product.price;
+        }
+        return value;
+    }
+}
+class Solution {
+    public static void callMethod() {
+        testCurrentStock();
+        testInventoryValue();
+        System.out.println("All tests passed.");
+    }
+    public static void testCurrentStock() {
+        InventoryManager manager = new InventoryManager();
+        manager.addProduct(
+                new Product(1, "Laptop", 50000.0)
+        );
+        manager.addMovement(
+                new InventoryMovement(
+                        1,
+                        MovementType.RESTOCK,
+                        10
+                )
+        );
+        manager.addMovement(
+                new InventoryMovement(
+                        1,
+                        MovementType.SALE,
+                        3
+                )
+        );
+        manager.addMovement(
+                new InventoryMovement(
+                        1,
+                        MovementType.RESTOCK,
+                        5
+                )
+        );
+        Assert.assertEquals(
+                12,
+                manager.getCurrentStock(1)
+        );
+    }
+    public static void testInventoryValue() {
+        InventoryManager manager = new InventoryManager();
+        manager.addProduct(
+                new Product(1, "Laptop", 50000.0)
+        );
+        manager.addProduct(
+                new Product(2, "Phone", 20000.0)
+        );
+        manager.addMovement(
+                new InventoryMovement(
+                        1,
+                        MovementType.RESTOCK,
+                        10
+                )
+        );
+        manager.addMovement(
+                new InventoryMovement(
+                        1,
+                        MovementType.SALE,
+                        4
+                )
+        );
+        manager.addMovement(
+                new InventoryMovement(
+                        2,
+                        MovementType.RESTOCK,
+                        5
+                )
+        );
+        Assert.assertEquals(
+                400000.0,
+                manager.getInventoryValue(),
+                0.0001
+        );
+    }
+}
+public class MainTest {
+    @Test
+    public void testMethod() {
+        Solution.callMethod();
     }
 }</t>
   </si>
@@ -451,7 +814,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -470,7 +833,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="360" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="277.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -478,7 +841,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
@@ -486,22 +849,45 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="302.39999999999998" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
+    </row>
+    <row r="5" spans="1:3" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C9" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>